<commit_message>
Update NewsPaperDeliverySystem User Stories and Acceptence Criteria.xlsx
</commit_message>
<xml_diff>
--- a/user stories/NewsPaperDeliverySystem User Stories and Acceptence Criteria.xlsx
+++ b/user stories/NewsPaperDeliverySystem User Stories and Acceptence Criteria.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5d60a861341b794a/Documents/GitHub/NewspaperDeliverySystem/user stories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EC1177F-EFC3-434C-B6CD-7E704E29B061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{7EC1177F-EFC3-434C-B6CD-7E704E29B061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7266095-2BC1-47AC-9309-D952ECA3A908}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{6307955D-1D03-43DF-8C9F-06C76E88F2E1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6307955D-1D03-43DF-8C9F-06C76E88F2E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="161">
   <si>
     <t>Number</t>
   </si>
@@ -77,9 +77,6 @@
     <t>to correct any mistakes.</t>
   </si>
   <si>
-    <t>Cu</t>
-  </si>
-  <si>
     <t>Verify entered user exists</t>
   </si>
   <si>
@@ -273,6 +270,264 @@
   </si>
   <si>
     <t>Verify the news agent not being able to restock the correct publication generates an errror message</t>
+  </si>
+  <si>
+    <t>Orders - User Stories</t>
+  </si>
+  <si>
+    <t>Order - AC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.As a news agent, </t>
+  </si>
+  <si>
+    <t>Verify the entered customer exists.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to place an order for newspapers to be delivered </t>
+  </si>
+  <si>
+    <t>Verify the entered publication exists.</t>
+  </si>
+  <si>
+    <t>as the customer has asked to receive newspapers regularly.</t>
+  </si>
+  <si>
+    <t>Verify the order ID is unique.</t>
+  </si>
+  <si>
+    <t>Verify the customer ID is not left empty.</t>
+  </si>
+  <si>
+    <t>Verify the publication ID is not left empty.</t>
+  </si>
+  <si>
+    <t>Verify a delivery pattern has been entered.</t>
+  </si>
+  <si>
+    <t>Verify the delivery pattern contains valid delivery days.</t>
+  </si>
+  <si>
+    <t>Verify the new order is successfully saved to the database.</t>
+  </si>
+  <si>
+    <t>Verify an invalid customer generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify an invalid publication generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify an empty customer ID generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify an empty publication ID generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify an invalid or empty delivery pattern generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify a duplicate order ID generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify the order not being successfully saved generates an error message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.As a news agent, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to be able to see what publications the customer is receiving </t>
+  </si>
+  <si>
+    <t>Verify the correct orders for the customer are retrieved.</t>
+  </si>
+  <si>
+    <t>because I want to remind myself of what publications they ordered.</t>
+  </si>
+  <si>
+    <t>Verify the correct publication ID is retrieved.</t>
+  </si>
+  <si>
+    <t>Verify the correct customer ID is retrieved.</t>
+  </si>
+  <si>
+    <t>Verify the correct delivery pattern is retrieved.</t>
+  </si>
+  <si>
+    <t>Verify only orders belonging to the entered customer are displayed.</t>
+  </si>
+  <si>
+    <t>Verify a customer with no existing orders generates an appropriate message.</t>
+  </si>
+  <si>
+    <t>Verify an order that does not exist generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify missing order information generates an error message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.As a news agent, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to update an order </t>
+  </si>
+  <si>
+    <t>Verify the entered order exists.</t>
+  </si>
+  <si>
+    <t>because a customer has changed their mind on what publication to receive.</t>
+  </si>
+  <si>
+    <t>Verify the newly entered publication exists.</t>
+  </si>
+  <si>
+    <t>Verify the delivery pattern is valid.</t>
+  </si>
+  <si>
+    <t>Verify the order remains associated with the correct customer.</t>
+  </si>
+  <si>
+    <t>Verify the order is successfully updated with the new information.</t>
+  </si>
+  <si>
+    <t>Verify a publication that does not exist generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify the order not being successfully updated generates an error message.</t>
+  </si>
+  <si>
+    <t>4.As a news agent,</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> I want to delete an order </t>
+  </si>
+  <si>
+    <t>as the customer accidentally ordered a publication.</t>
+  </si>
+  <si>
+    <t>Verify the order belongs to the entered customer.</t>
+  </si>
+  <si>
+    <t>Verify the correct order is successfully deleted from the database.</t>
+  </si>
+  <si>
+    <t>Verify the deleted order can no longer be retrieved.</t>
+  </si>
+  <si>
+    <t>Verify the customer remains in the database after the order is deleted.</t>
+  </si>
+  <si>
+    <t>Verify an order belonging to another customer cannot be deleted.</t>
+  </si>
+  <si>
+    <t>Verify the order not being successfully deleted generates an error message.</t>
+  </si>
+  <si>
+    <t>Customer - US</t>
+  </si>
+  <si>
+    <t>Cust - AC</t>
+  </si>
+  <si>
+    <t>Verify the customer ID is unique.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to create a new customer </t>
+  </si>
+  <si>
+    <t>Verify the customer name is not left empty.</t>
+  </si>
+  <si>
+    <t>because a new local customer wants me to deliver newspapers.</t>
+  </si>
+  <si>
+    <t>Verify the customer name has a minimum of 1 character.</t>
+  </si>
+  <si>
+    <t>Verify the customer address is not left empty.</t>
+  </si>
+  <si>
+    <t>Verify the customer contact details are not left empty.</t>
+  </si>
+  <si>
+    <t>Verify the new customer is successfully saved to the database.</t>
+  </si>
+  <si>
+    <t>Verify an empty name field generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify an empty address field generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify empty contact details generate an error message.</t>
+  </si>
+  <si>
+    <t>Verify a duplicate customer ID generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify the customer not being successfully saved generates an error message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to update a customer's details </t>
+  </si>
+  <si>
+    <t>so that any deliveries are delivered to them correctly.</t>
+  </si>
+  <si>
+    <t>Verify the customer's details are successfully updated in the database.</t>
+  </si>
+  <si>
+    <t>Verify a customer that does not exist generates an error message.</t>
+  </si>
+  <si>
+    <t>Verify the customer not being successfully updated generates an error message.</t>
+  </si>
+  <si>
+    <t>3.As a news agent,</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> I want to be able to see a customer's details </t>
+  </si>
+  <si>
+    <t>Verify the correct customer is retrieved.</t>
+  </si>
+  <si>
+    <t>to ensure if they are correct.</t>
+  </si>
+  <si>
+    <t>Verify the customer ID is retrieved.</t>
+  </si>
+  <si>
+    <t>Verify the customer's name is retrieved.</t>
+  </si>
+  <si>
+    <t>Verify the customer's address is retrieved.</t>
+  </si>
+  <si>
+    <t>Verify the customer's contact details are retrieved.</t>
+  </si>
+  <si>
+    <t>Verify missing customer details generate an error message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.As a news agent, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to delete a customer's account </t>
+  </si>
+  <si>
+    <t>Verify the correct customer is selected for deletion.</t>
+  </si>
+  <si>
+    <t>as they no longer wish to receive newspapers regularly.</t>
+  </si>
+  <si>
+    <t>Verify the customer is successfully deleted from the database.</t>
+  </si>
+  <si>
+    <t>Verify the deleted customer can no longer be retrieved.</t>
+  </si>
+  <si>
+    <t>Verify the customer not being successfully deleted generates an error message.</t>
   </si>
 </sst>
 </file>
@@ -648,13 +903,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6669703-D861-4853-A03C-2BD7E616836D}">
   <dimension ref="A1:C34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="49" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -665,7 +920,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -673,61 +928,61 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>7</v>
       </c>
       <c r="C4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C6" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2</v>
       </c>
@@ -735,31 +990,31 @@
         <v>3</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3</v>
       </c>
@@ -767,51 +1022,51 @@
         <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>9</v>
       </c>
       <c r="C21" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C22" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C23" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C26" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>4</v>
       </c>
@@ -819,38 +1074,38 @@
         <v>3</v>
       </c>
       <c r="C29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B30" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
         <v>21</v>
       </c>
-      <c r="C30" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>22</v>
       </c>
-      <c r="C31" t="s">
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C32" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -860,21 +1115,521 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC1FDFD2-DDDE-4B64-B452-BAE227FEA908}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A1:B52"/>
+  <sheetFormatPr defaultColWidth="77.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>106</v>
+      </c>
+      <c r="B30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>107</v>
+      </c>
+      <c r="B31" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>109</v>
+      </c>
+      <c r="B32" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>116</v>
+      </c>
+      <c r="B43" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>117</v>
+      </c>
+      <c r="B44" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>118</v>
+      </c>
+      <c r="B45" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>124</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBA3C9B1-67AE-4FC3-9A3C-0CAB1ECF3271}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B40"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="65.42578125" customWidth="1"/>
+    <col min="2" max="2" width="71.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>125</v>
+      </c>
+      <c r="B1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>141</v>
+      </c>
+      <c r="B17" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>145</v>
+      </c>
+      <c r="B26" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>146</v>
+      </c>
+      <c r="B27" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>148</v>
+      </c>
+      <c r="B28" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>154</v>
+      </c>
+      <c r="B35" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>155</v>
+      </c>
+      <c r="B36" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>157</v>
+      </c>
+      <c r="B37" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -885,13 +1640,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D878139E-7EB3-4925-9F6E-43018AC46F66}">
   <dimension ref="A1:C50"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="85.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="85.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -902,274 +1657,274 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
         <v>34</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C5" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C12" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C13" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C14" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C15" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>3</v>
       </c>
       <c r="C17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B18" t="s">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
         <v>36</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>3</v>
       </c>
       <c r="C22" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B23" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B24" t="s">
-        <v>39</v>
-      </c>
-      <c r="C24" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C25" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C26" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C27" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C28" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C29" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C30" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C31" t="s">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C32" t="s">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C33" t="s">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C34" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C34" t="s">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C35" t="s">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C36" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C36" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>3</v>
       </c>
       <c r="C38" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
+        <v>39</v>
+      </c>
+      <c r="C39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
         <v>40</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C40" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B40" t="s">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
         <v>41</v>
       </c>
-      <c r="C40" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C41" t="s">
+      <c r="C43" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>42</v>
+      </c>
+      <c r="C44" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>43</v>
+      </c>
+      <c r="C45" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B43" t="s">
-        <v>42</v>
-      </c>
-      <c r="C43" t="s">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C46" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C47" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B44" t="s">
-        <v>43</v>
-      </c>
-      <c r="C44" t="s">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C48" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B45" t="s">
-        <v>44</v>
-      </c>
-      <c r="C45" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C46" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C47" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C48" t="s">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C49" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C49" t="s">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C50" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C50" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1180,7 +1935,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC3B0FF-370B-4D26-9C5F-A03D18CBAD5F}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1189,7 +1944,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74CBA472-5F67-4E03-9BD0-AEC7A8404DF5}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1198,7 +1953,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{976F6F6C-4BF2-4009-9A4D-82FF59E3879F}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>